<commit_message>
last commit before gerber export
</commit_message>
<xml_diff>
--- a/charging_controller/Hardware/reference/Charging_controller_BOM.xlsx
+++ b/charging_controller/Hardware/reference/Charging_controller_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asiadel\Documents\FIRO\firo_electronics\charging_controller\Hardware\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3A4EB8-6832-4CFF-BAB2-EC96ED0973FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEC7A25-BB94-4770-966B-05F8BB017933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -551,7 +551,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -562,7 +562,6 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
@@ -590,6 +589,8 @@
     <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="2" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperłącze" xfId="2" builtinId="8"/>
@@ -947,28 +948,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="20"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -992,13 +993,13 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="16" t="s">
         <v>40</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="37" t="s">
         <v>48</v>
       </c>
       <c r="D3" s="7">
@@ -1016,7 +1017,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -1040,13 +1041,13 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="16" t="s">
         <v>41</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="37" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="7">
@@ -1064,26 +1065,26 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="16" t="s">
         <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="34">
         <v>54.3</v>
       </c>
-      <c r="E6" s="36">
-        <v>1</v>
-      </c>
-      <c r="F6" s="37">
+      <c r="E6" s="35">
+        <v>1</v>
+      </c>
+      <c r="F6" s="36">
         <f t="shared" si="0"/>
         <v>54.3</v>
       </c>
-      <c r="G6" s="36" t="s">
+      <c r="G6" s="35" t="s">
         <v>6</v>
       </c>
       <c r="H6" t="s">
@@ -1091,13 +1092,13 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="16" t="s">
         <v>50</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="37" t="s">
         <v>52</v>
       </c>
       <c r="D7" s="7">
@@ -1115,22 +1116,22 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>68</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="10">
         <v>0.35299999999999998</v>
       </c>
       <c r="E8" s="9">
         <v>1</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="11">
         <f t="shared" si="0"/>
         <v>0.35299999999999998</v>
       </c>
@@ -1139,22 +1140,22 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="17" t="s">
         <v>71</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="10">
         <v>0.27500000000000002</v>
       </c>
       <c r="E9" s="9">
         <v>1</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="11">
         <f t="shared" si="0"/>
         <v>0.27500000000000002</v>
       </c>
@@ -1163,22 +1164,22 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>74</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="10">
         <v>0.75</v>
       </c>
       <c r="E10" s="9">
         <v>1</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="11">
         <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
@@ -1187,22 +1188,22 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="10">
         <v>9.4E-2</v>
       </c>
       <c r="E11" s="9">
         <v>1</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="11">
         <f t="shared" ref="F11" si="1">D11*E11</f>
         <v>9.4E-2</v>
       </c>
@@ -1211,22 +1212,22 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="17" t="s">
         <v>80</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="10">
         <v>0.68899999999999995</v>
       </c>
       <c r="E12" s="9">
         <v>1</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="11">
         <f t="shared" ref="F12" si="2">D12*E12</f>
         <v>0.68899999999999995</v>
       </c>
@@ -1235,349 +1236,349 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="14">
         <v>0.159</v>
       </c>
-      <c r="E13" s="13">
-        <v>1</v>
-      </c>
-      <c r="F13" s="16">
-        <f>D13*E13</f>
+      <c r="E13" s="12">
+        <v>1</v>
+      </c>
+      <c r="F13" s="15">
+        <f t="shared" ref="F13:F18" si="3">D13*E13</f>
         <v>0.159</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="12">
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="12">
         <v>9</v>
       </c>
-      <c r="F14" s="16">
-        <f>D14*E14</f>
+      <c r="F14" s="15">
+        <f t="shared" si="3"/>
         <v>0.432</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="14">
         <v>0.121</v>
       </c>
-      <c r="E15" s="13">
-        <v>1</v>
-      </c>
-      <c r="F15" s="16">
-        <f>D15*E15</f>
+      <c r="E15" s="12">
+        <v>1</v>
+      </c>
+      <c r="F15" s="15">
+        <f t="shared" si="3"/>
         <v>0.121</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="G15" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="14">
         <v>0.126</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="12">
         <v>2</v>
       </c>
-      <c r="F16" s="16">
-        <f>D16*E16</f>
+      <c r="F16" s="15">
+        <f t="shared" si="3"/>
         <v>0.252</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="14">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="E17" s="13">
-        <v>1</v>
-      </c>
-      <c r="F17" s="16">
-        <f>D17*E17</f>
+      <c r="E17" s="12">
+        <v>1</v>
+      </c>
+      <c r="F17" s="15">
+        <f t="shared" si="3"/>
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="14">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="12">
         <v>2</v>
       </c>
-      <c r="F18" s="16">
-        <f>D18*E18</f>
+      <c r="F18" s="15">
+        <f t="shared" si="3"/>
         <v>5.8000000000000003E-2</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="14">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="12">
         <v>2</v>
       </c>
-      <c r="F19" s="16">
-        <f t="shared" ref="F19" si="3">D19*E19</f>
+      <c r="F19" s="15">
+        <f t="shared" ref="F19" si="4">D19*E19</f>
         <v>0.17799999999999999</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="G19" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="33" t="s">
+      <c r="C20" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="14">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="12">
         <v>2</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="15">
         <f>D20*E20</f>
         <v>0.17599999999999999</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="G20" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="14">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E21" s="13">
-        <v>1</v>
-      </c>
-      <c r="F21" s="16">
+      <c r="E21" s="12">
+        <v>1</v>
+      </c>
+      <c r="F21" s="15">
         <f>D21*E21</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="33" t="s">
+      <c r="C22" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="14">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="E22" s="13">
-        <v>2</v>
-      </c>
-      <c r="F22" s="16">
+      <c r="E22" s="12">
+        <v>3</v>
+      </c>
+      <c r="F22" s="15">
         <f>D22*E22</f>
-        <v>0.05</v>
-      </c>
-      <c r="G22" s="13" t="s">
+        <v>7.5000000000000011E-2</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="C23" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="14">
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="E23" s="13">
-        <v>1</v>
-      </c>
-      <c r="F23" s="16">
+      <c r="E23" s="12">
+        <v>1</v>
+      </c>
+      <c r="F23" s="15">
         <f>D23*E23</f>
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="33" t="s">
+      <c r="C24" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="14">
         <v>4.7E-2</v>
       </c>
-      <c r="E24" s="13">
-        <v>1</v>
-      </c>
-      <c r="F24" s="16">
-        <f t="shared" ref="F24:F25" si="4">D24*E24</f>
+      <c r="E24" s="12">
+        <v>1</v>
+      </c>
+      <c r="F24" s="15">
+        <f t="shared" ref="F24:F25" si="5">D24*E24</f>
         <v>4.7E-2</v>
       </c>
-      <c r="G24" s="13" t="s">
+      <c r="G24" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C25" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="14">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="E25" s="13">
+      <c r="E25" s="12">
         <v>3</v>
       </c>
-      <c r="F25" s="16">
-        <f t="shared" si="4"/>
+      <c r="F25" s="15">
+        <f t="shared" si="5"/>
         <v>0.153</v>
       </c>
-      <c r="G25" s="13" t="s">
+      <c r="G25" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="C26" s="33" t="s">
+      <c r="C26" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="14">
         <v>2.7E-2</v>
       </c>
-      <c r="E26" s="13">
+      <c r="E26" s="12">
         <v>2</v>
       </c>
-      <c r="F26" s="16">
-        <f t="shared" ref="F26" si="5">D26*E26</f>
+      <c r="F26" s="15">
+        <f t="shared" ref="F26" si="6">D26*E26</f>
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="28" t="s">
         <v>98</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="29" t="s">
         <v>100</v>
       </c>
       <c r="D27" s="2">
@@ -1587,7 +1588,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="3">
-        <f>D27*E27</f>
+        <f t="shared" ref="F27:F33" si="7">D27*E27</f>
         <v>0.52600000000000002</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -1595,13 +1596,13 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="28" t="s">
         <v>86</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="C28" s="29" t="s">
         <v>87</v>
       </c>
       <c r="D28" s="2">
@@ -1611,7 +1612,7 @@
         <v>1</v>
       </c>
       <c r="F28" s="3">
-        <f>D28*E28</f>
+        <f t="shared" si="7"/>
         <v>0.78800000000000003</v>
       </c>
       <c r="G28" s="1" t="s">
@@ -1619,13 +1620,13 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="28" t="s">
         <v>89</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C29" s="30" t="s">
+      <c r="C29" s="29" t="s">
         <v>91</v>
       </c>
       <c r="D29" s="2">
@@ -1635,7 +1636,7 @@
         <v>1</v>
       </c>
       <c r="F29" s="3">
-        <f>D29*E29</f>
+        <f t="shared" si="7"/>
         <v>0.495</v>
       </c>
       <c r="G29" s="1" t="s">
@@ -1643,13 +1644,13 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="28" t="s">
         <v>92</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="29" t="s">
         <v>96</v>
       </c>
       <c r="D30" s="2">
@@ -1659,7 +1660,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="3">
-        <f>D30*E30</f>
+        <f t="shared" si="7"/>
         <v>0.59799999999999998</v>
       </c>
       <c r="G30" s="1" t="s">
@@ -1667,13 +1668,13 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="28" t="s">
         <v>93</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="29" t="s">
         <v>97</v>
       </c>
       <c r="D31" s="2">
@@ -1683,7 +1684,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="3">
-        <f>D31*E31</f>
+        <f t="shared" si="7"/>
         <v>0.56799999999999995</v>
       </c>
       <c r="G31" s="1" t="s">
@@ -1691,13 +1692,13 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="29" t="s">
+      <c r="A32" s="28" t="s">
         <v>111</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="29" t="s">
         <v>113</v>
       </c>
       <c r="D32" s="2">
@@ -1707,7 +1708,7 @@
         <v>2</v>
       </c>
       <c r="F32" s="3">
-        <f>D32*E32</f>
+        <f t="shared" si="7"/>
         <v>9.5</v>
       </c>
       <c r="G32" s="1" t="s">
@@ -1715,13 +1716,13 @@
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="28" t="s">
         <v>114</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="29" t="s">
         <v>116</v>
       </c>
       <c r="D33" s="2">
@@ -1731,7 +1732,7 @@
         <v>1</v>
       </c>
       <c r="F33" s="3">
-        <f>D33*E33</f>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
       <c r="G33" s="1" t="s">
@@ -1739,13 +1740,13 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" s="29" t="s">
+      <c r="A34" s="28" t="s">
         <v>117</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="29" t="s">
         <v>116</v>
       </c>
       <c r="D34" s="2">
@@ -1755,7 +1756,7 @@
         <v>3</v>
       </c>
       <c r="F34" s="3">
-        <f t="shared" ref="F34:F35" si="6">D34*E34</f>
+        <f t="shared" ref="F34" si="8">D34*E34</f>
         <v>14.97</v>
       </c>
       <c r="G34" s="1" t="s">
@@ -1763,107 +1764,107 @@
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="B35" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="25" t="s">
+      <c r="C35" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="D35" s="24">
+      <c r="D35" s="23">
         <v>0.16800000000000001</v>
       </c>
-      <c r="E35" s="22">
+      <c r="E35" s="21">
         <v>2</v>
       </c>
-      <c r="F35" s="23">
+      <c r="F35" s="22">
         <f>D35*E35</f>
         <v>0.33600000000000002</v>
       </c>
-      <c r="G35" s="22" t="s">
+      <c r="G35" s="21" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="25" t="s">
+      <c r="C36" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="D36" s="24">
+      <c r="D36" s="23">
         <v>0.125</v>
       </c>
-      <c r="E36" s="22">
+      <c r="E36" s="21">
         <v>3</v>
       </c>
-      <c r="F36" s="23">
-        <f t="shared" ref="F36:F37" si="7">D36*E36</f>
+      <c r="F36" s="22">
+        <f t="shared" ref="F36:F37" si="9">D36*E36</f>
         <v>0.375</v>
       </c>
-      <c r="G36" s="22" t="s">
+      <c r="G36" s="21" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="32" t="s">
+      <c r="C37" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="31">
+      <c r="D37" s="30">
         <v>0.82799999999999996</v>
       </c>
-      <c r="E37" s="26">
-        <v>1</v>
-      </c>
-      <c r="F37" s="27">
-        <f t="shared" si="7"/>
+      <c r="E37" s="25">
+        <v>1</v>
+      </c>
+      <c r="F37" s="26">
+        <f t="shared" si="9"/>
         <v>0.82799999999999996</v>
       </c>
-      <c r="G37" s="26" t="s">
+      <c r="G37" s="25" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="C38" s="32" t="s">
+      <c r="C38" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="D38" s="31">
+      <c r="D38" s="30">
         <v>0.33400000000000002</v>
       </c>
-      <c r="E38" s="26">
-        <v>1</v>
-      </c>
-      <c r="F38" s="27">
-        <f t="shared" ref="F38" si="8">D38*E38</f>
+      <c r="E38" s="25">
+        <v>1</v>
+      </c>
+      <c r="F38" s="26">
+        <f t="shared" ref="F38" si="10">D38*E38</f>
         <v>0.33400000000000002</v>
       </c>
-      <c r="G38" s="26" t="s">
+      <c r="G38" s="25" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F39" s="4">
         <f>SUM(F2:F5,F7:F38)</f>
-        <v>51.494999999999997</v>
-      </c>
-      <c r="G39" s="34" t="s">
+        <v>51.519999999999996</v>
+      </c>
+      <c r="G39" s="33" t="s">
         <v>6</v>
       </c>
       <c r="H39" t="s">
@@ -1887,6 +1888,15 @@
     <hyperlink ref="C23" r:id="rId12" xr:uid="{5AF84C12-E9B6-422B-806D-4571FEA3B881}"/>
     <hyperlink ref="C17" r:id="rId13" xr:uid="{9A10AD12-C8C7-474E-9ED2-29EF87197BB9}"/>
     <hyperlink ref="C16" r:id="rId14" xr:uid="{A8304D9E-AB1A-47A3-81D7-ABB852029660}"/>
+    <hyperlink ref="C3" r:id="rId15" xr:uid="{23125A78-972C-4C3F-B9A3-B80C51FF0F4D}"/>
+    <hyperlink ref="C5" r:id="rId16" xr:uid="{67E61E1E-6221-4840-852A-453291729FD7}"/>
+    <hyperlink ref="C6" r:id="rId17" xr:uid="{34B453A5-1DA4-43B2-98FA-EA23A54F6360}"/>
+    <hyperlink ref="C7" r:id="rId18" xr:uid="{72A0C805-AF6C-4461-9030-76995966144F}"/>
+    <hyperlink ref="C8" r:id="rId19" xr:uid="{6CBB2834-2782-4756-93C3-63DF46857950}"/>
+    <hyperlink ref="C9" r:id="rId20" xr:uid="{50EF1C27-80E8-4EC1-B2FC-26CEBC716AFE}"/>
+    <hyperlink ref="C10" r:id="rId21" xr:uid="{C89155AB-454A-45F9-8858-7E9E762016AE}"/>
+    <hyperlink ref="C12" r:id="rId22" xr:uid="{C8CF260F-3E00-45F4-B815-BA5D67CF0545}"/>
+    <hyperlink ref="C27" r:id="rId23" xr:uid="{98B5BC2C-B60B-41D2-986F-165AAD06D42F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>